<commit_message>
Update human validation files: enhance README with third-rater QA process details, remove outdated PDF files, and update CSV and Excel sheets for improved data management.
</commit_message>
<xml_diff>
--- a/results/human_validation/ft_qa_extraction_blind_review_sheet.xlsx
+++ b/results/human_validation/ft_qa_extraction_blind_review_sheet.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD178"/>
+  <dimension ref="A1:AD180"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="11.33203125" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -674,7 +674,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>exclude</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0079_a_framework_for_measuring_the_quality_of_business_pr.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0079_a_framework_for_measuring_the_quality_of_business_pr.pdf</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0003_a_note_on_two_stage_software_testing_by_two_teams.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0003_a_note_on_two_stage_software_testing_by_two_teams.pdf</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -794,6 +794,11 @@
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -853,6 +858,16 @@
           <t>chapter</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="6" hidden="1" ht="16" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -900,6 +915,16 @@
           <t>article</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="7" hidden="1" ht="256" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -939,7 +964,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0014_detection_and_correction_process_modeling_considerin.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0014_detection_and_correction_process_modeling_considerin.pdf</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -950,6 +975,11 @@
       <c r="K7" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -991,7 +1021,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0047_process_discovery_automated_approach_for_block_disco.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0047_process_discovery_automated_approach_for_block_disco.pdf</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1002,6 +1032,11 @@
       <c r="K8" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1026,6 +1061,11 @@
           <t>This paper proposes an advanced, open architecture to augment streaming data platforms with both complex event processing (CEP) and predictive machine learning models. We leverage the power of CEP to preprocess streams using sophisticated event pattern expressions then present these preprocessed streams for downstream training and predictive computations. We demonstrate this approach using specific technology components</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>10.1109/EDOC49727.2020.00016</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>https://www.scopus.com/record/display.uri?eid=2-s2.0-85096558116</t>
@@ -1033,7 +1073,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0069_proceedings_2020_ieee_24th_international_enterprise.pdf</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1044,6 +1084,16 @@
       <c r="K9" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>PDF encontrado via snowballing; DOI confirmado no rodape do PDF (nao estava na planilha original, que so tinha o titulo do proceedings via Scopus).</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1130,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0148_an_intelligent_methodology_to_enhance_requirements.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0148_an_intelligent_methodology_to_enhance_requirements.pdf</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1091,6 +1141,11 @@
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1187,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0012_modeling_and_predicting_software_failure_costs.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0012_modeling_and_predicting_software_failure_costs.pdf</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1143,6 +1198,11 @@
       <c r="K11" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1244,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0124_use_of_combined_system_dependability_and_software_re.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0124_use_of_combined_system_dependability_and_software_re.pdf</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1195,6 +1255,11 @@
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1301,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0052_extension_of_a_simulation_software_to_incorporate_qu.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0052_extension_of_a_simulation_software_to_incorporate_qu.pdf</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1247,6 +1312,11 @@
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1353,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0164_intervention_of_knowledge_flows_in_software_proces.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0164_intervention_of_knowledge_flows_in_software_proces.pdf</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1294,6 +1364,11 @@
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1410,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0130_online_discovery_of_simulation_models_for_evolving.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0130_online_discovery_of_simulation_models_for_evolving.pdf</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1346,6 +1421,11 @@
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1467,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0035_software_reliability_estimation_method_based_on_mark.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0035_software_reliability_estimation_method_based_on_mark.pdf</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1398,6 +1478,11 @@
       <c r="K16" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1452,9 +1537,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1581,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0175_process_mining_software_repositories_from_student_pr.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0175_process_mining_software_repositories_from_student_pr.pdf</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1502,6 +1592,11 @@
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1546,9 +1641,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -1603,9 +1703,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1757,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0096_cutting_the_software_building_efforts_in_continuou.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0096_cutting_the_software_building_efforts_in_continuou.pdf</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1663,6 +1768,11 @@
       <c r="K21" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1819,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0065_representing_software_usage_models_with_stochastic_a.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0065_representing_software_usage_models_with_stochastic_a.pdf</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1720,6 +1830,11 @@
       <c r="K22" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1881,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0086_software_reliability_assessment_an_architectural_and.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0086_software_reliability_assessment_an_architectural_and.pdf</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1777,6 +1892,11 @@
       <c r="K23" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1938,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0006_generating_event_logs_with_workload_dependent_speeds.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0006_generating_event_logs_with_workload_dependent_speeds.pdf</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1829,6 +1949,11 @@
       <c r="K24" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1990,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0134_petri_nets_simulation_for_operational_analytics_base.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0134_petri_nets_simulation_for_operational_analytics_base.pdf</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -1876,6 +2001,11 @@
       <c r="K25" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -1912,7 +2042,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0133_reusing_simulation_experiment_specifications_to_supp.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0133_reusing_simulation_experiment_specifications_to_supp.pdf</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -1923,6 +2053,11 @@
       <c r="K26" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -1962,9 +2097,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>no access file, no abstract, no title</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2141,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0156_supporting_software_evolution_actions_with_process.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0156_supporting_software_evolution_actions_with_process.pdf</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2012,6 +2152,11 @@
       <c r="K28" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2203,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0110_combination_of_process_mining_and_simulation_techn.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0110_combination_of_process_mining_and_simulation_techn.pdf</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2069,6 +2214,11 @@
       <c r="K29" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2260,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0095_model_driven_safety_modeling_and_analysis_of_embedde.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0095_model_driven_safety_modeling_and_analysis_of_embedde.pdf</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2121,6 +2271,11 @@
       <c r="K30" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2322,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0131_a_stratification_and_sampling_model_for_bellwether.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0131_a_stratification_and_sampling_model_for_bellwether.pdf</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2178,6 +2333,11 @@
       <c r="K31" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2384,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0018_distributed_process_discovery_and_conformance_chec.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0018_distributed_process_discovery_and_conformance_chec.pdf</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2235,6 +2395,11 @@
       <c r="K32" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2446,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0162_unearthing_open_source_decision_making_processes_a.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0162_unearthing_open_source_decision_making_processes_a.pdf</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -2292,6 +2457,11 @@
       <c r="K33" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2503,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0135_software_reliability_considering_the_superposition_o.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0135_software_reliability_considering_the_superposition_o.pdf</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2344,6 +2514,11 @@
       <c r="K34" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2576,12 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>no ok - discard</t>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>discard (motivo original: no ok - discard)</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2623,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0147_devops_workflow_verification_and_duration_predicti.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0147_devops_workflow_verification_and_duration_predicti.pdf</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2454,6 +2634,11 @@
       <c r="K36" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2680,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0099_an_empirical_study_of_the_evolution_of_github_acti.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0099_an_empirical_study_of_the_evolution_of_github_acti.pdf</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2506,6 +2691,11 @@
       <c r="K37" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2737,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0060_an_iterative_decision_making_scheme_for_markov_decis.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0060_an_iterative_decision_making_scheme_for_markov_decis.pdf</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2558,6 +2748,11 @@
       <c r="K38" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2794,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0078_mining_constraints_for_event_based_monitoring_in_sys.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0078_mining_constraints_for_event_based_monitoring_in_sys.pdf</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -2610,6 +2805,11 @@
       <c r="K39" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2649,9 +2849,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>no access file, no abstract, no title</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2903,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0161_probabilistic_model_checking_github_repositories_f.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0161_probabilistic_model_checking_github_repositories_f.pdf</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -2709,6 +2914,11 @@
       <c r="K41" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2748,9 +2958,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>no access file, no abstract, no title</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -2790,11 +3005,7 @@
           <t>https://www.scopus.com/record/display.uri?eid=2-s2.0-85077113635</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0136_formal_modeling_and_analysis_of_probabilistic_real_t.pdf</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr">
         <is>
           <t>Advances in Intelligent Systems and Computing</t>
@@ -2803,6 +3014,11 @@
       <c r="K43" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
@@ -2839,7 +3055,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0072_a_stochastic_approach_to_security_software_quality_m.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0072_a_stochastic_approach_to_security_software_quality_m.pdf</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -2850,6 +3066,11 @@
       <c r="K44" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2899,9 +3120,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -2938,7 +3164,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0002_leveraging_process_mining_techniques_for_up_to_date.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0002_leveraging_process_mining_techniques_for_up_to_date.pdf</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -2949,6 +3175,11 @@
       <c r="K46" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -2990,7 +3221,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0051_software_process_simulation_modeling_preliminary_res.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0051_software_process_simulation_modeling_preliminary_res.pdf</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -3001,6 +3232,11 @@
       <c r="K47" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3283,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0100_better_reasoning_about_software_engineering_activi.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0100_better_reasoning_about_software_engineering_activi.pdf</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -3058,6 +3294,11 @@
       <c r="K48" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -3112,9 +3353,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3402,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0158_probabilistic_approach_to_predicting_risk_in_softw.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0158_probabilistic_approach_to_predicting_risk_in_softw.pdf</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3167,6 +3413,11 @@
       <c r="K50" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3203,7 +3454,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0172_mining_software_process_lines.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0172_mining_software_process_lines.pdf</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -3214,6 +3465,11 @@
       <c r="K51" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3506,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0090_discrete_and_continuous_time_high_order_markov_mod.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0090_discrete_and_continuous_time_high_order_markov_mod.pdf</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -3261,6 +3517,11 @@
       <c r="K52" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3558,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0159_experiences_in_discovering_modeling_and_reenacting_o.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0159_experiences_in_discovering_modeling_and_reenacting_o.pdf</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -3308,6 +3569,11 @@
       <c r="K53" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -3349,7 +3615,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0125_software_safety_assessment_based_on_a_subordinated_m.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0125_software_safety_assessment_based_on_a_subordinated_m.pdf</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3360,6 +3626,11 @@
       <c r="K54" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3672,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0007_mining_issue_trackers_concepts_and_techniques.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0007_mining_issue_trackers_concepts_and_techniques.pdf</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -3412,6 +3683,11 @@
       <c r="K55" s="2" t="inlineStr">
         <is>
           <t>chapter</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3729,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0010_systematic_mapping_study_on_process_mining_in_agile.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0010_systematic_mapping_study_on_process_mining_in_agile.pdf</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -3464,6 +3740,11 @@
       <c r="K56" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3513,9 +3794,14 @@
           <t>editorial</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3838,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0075_probabilistic_learning_of_temporal_uncertainties_in.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0075_probabilistic_learning_of_temporal_uncertainties_in.pdf</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3563,6 +3849,11 @@
       <c r="K58" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3900,7 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0087_holistic_discovery_of_decision_models_from_process.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0087_holistic_discovery_of_decision_models_from_process.pdf</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
@@ -3620,6 +3911,11 @@
       <c r="K59" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3664,9 +3960,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -3708,7 +4009,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0019_bayesian_inference_for_nonhomogeneous_poisson_proces.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0019_bayesian_inference_for_nonhomogeneous_poisson_proces.pdf</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -3719,6 +4020,11 @@
       <c r="K61" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3755,7 +4061,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0115_towards_automated_conformance_checking_of_ebbp_st_ch.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0115_towards_automated_conformance_checking_of_ebbp_st_ch.pdf</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -3766,6 +4072,11 @@
       <c r="K62" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -3807,7 +4118,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0091_characterization_of_operational_failures_from_a_busi.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0091_characterization_of_operational_failures_from_a_busi.pdf</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
@@ -3818,6 +4129,11 @@
       <c r="K63" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3859,7 +4175,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0144_analysis_of_software_repositories_using_process_mini.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0144_analysis_of_software_repositories_using_process_mini.pdf</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -3870,6 +4186,11 @@
       <c r="K64" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3916,7 +4237,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0037_reducing_user_input_requests_to_improve_it_support.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0037_reducing_user_input_requests_to_improve_it_support.pdf</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -3927,6 +4248,11 @@
       <c r="K65" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -3973,7 +4299,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0154_business_process_analysis_of_programmer_job_role_in.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0154_business_process_analysis_of_programmer_job_role_in.pdf</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -3984,6 +4310,11 @@
       <c r="K66" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4361,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0033_assessing_process_centered_software_engineering_envi.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0033_assessing_process_centered_software_engineering_envi.pdf</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -4041,6 +4372,11 @@
       <c r="K67" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -4095,9 +4431,14 @@
           <t>article</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4480,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0103_extending_hybrid_csp_with_probability_and_stochast.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0103_extending_hybrid_csp_with_probability_and_stochast.pdf</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -4150,6 +4491,11 @@
       <c r="K69" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4537,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0088_ssrgm_software_strong_reliability_growth_model_based.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0088_ssrgm_software_strong_reliability_growth_model_based.pdf</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -4202,6 +4548,11 @@
       <c r="K70" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4233,7 +4584,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0049_towards_organizational_digital_twins_process_enhance.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0049_towards_organizational_digital_twins_process_enhance.pdf</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -4244,6 +4595,11 @@
       <c r="K71" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4285,7 +4641,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0085_model_based_scheduling_analysis_for_software_project.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0085_model_based_scheduling_analysis_for_software_project.pdf</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -4296,6 +4652,11 @@
       <c r="K72" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4327,7 +4688,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0004_data_driven_simulation_based_analysis_of_collaborati.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0004_data_driven_simulation_based_analysis_of_collaborati.pdf</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -4338,6 +4699,11 @@
       <c r="K73" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4384,7 +4750,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0123_uncertainty_risk_and_information_value_in_software.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0123_uncertainty_risk_and_information_value_in_software.pdf</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4395,6 +4761,11 @@
       <c r="K74" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4807,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0176_an_exploratory_study_of_process_enactment_as_input_t.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0176_an_exploratory_study_of_process_enactment_as_input_t.pdf</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4447,6 +4818,11 @@
       <c r="K75" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4501,6 +4877,16 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="88" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
@@ -4553,9 +4939,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4988,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0059_arch_comp25_category_report_stochastic_models.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0059_arch_comp25_category_report_stochastic_models.pdf</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4608,6 +4999,11 @@
       <c r="K78" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4649,7 +5045,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0045_a_hybrid_process_mining_approach_for_simulation_mode.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0045_a_hybrid_process_mining_approach_for_simulation_mode.pdf</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -4660,6 +5056,11 @@
       <c r="K79" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4701,7 +5102,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0076_cosmo_a_framework_to_instantiate_conditioned_proce.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0076_cosmo_a_framework_to_instantiate_conditioned_proce.pdf</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -4712,6 +5113,11 @@
       <c r="K80" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4751,9 +5157,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -4793,9 +5204,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -4837,7 +5253,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0008_modeling_the_failure_pathology_of_software_component.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0008_modeling_the_failure_pathology_of_software_component.pdf</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -4848,6 +5264,11 @@
       <c r="K83" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -4879,7 +5300,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0068_special_panel_software_process_simulation_at_a_cross.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0068_special_panel_software_process_simulation_at_a_cross.pdf</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4890,6 +5311,11 @@
       <c r="K84" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -4929,9 +5355,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M85" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -4973,7 +5404,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0038_software_reliability.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0038_software_reliability.pdf</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -4984,6 +5415,11 @@
       <c r="K86" s="2" t="inlineStr">
         <is>
           <t>review</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
       <c r="M86" s="2" t="inlineStr">
@@ -5035,7 +5471,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0107_software_reliability_test_case_generation_using_temp.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0107_software_reliability_test_case_generation_using_temp.pdf</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -5046,6 +5482,11 @@
       <c r="K87" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5533,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0138_microflows_enabling_agile_business_process_modeling.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0138_microflows_enabling_agile_business_process_modeling.pdf</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -5103,6 +5544,11 @@
       <c r="K88" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5149,7 +5595,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0102_guiding_the_discovery_of_open_source_software_proc.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0102_guiding_the_discovery_of_open_source_software_proc.pdf</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -5160,6 +5606,11 @@
       <c r="K89" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5652,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0025_gitprojecthealth_an_extensible_framework_for_git_soc.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0025_gitprojecthealth_an_extensible_framework_for_git_soc.pdf</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -5212,6 +5663,11 @@
       <c r="K90" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5709,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0169_an_integrated_infrastructure_using_process_mining_te.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0169_an_integrated_infrastructure_using_process_mining_te.pdf</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -5264,6 +5720,11 @@
       <c r="K91" s="2" t="inlineStr">
         <is>
           <t>chapter</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5303,6 +5764,16 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="93" hidden="1" ht="160" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
@@ -5342,7 +5813,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0043_predicting_data_access_patterns_in_object_oriented_a.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0043_predicting_data_access_patterns_in_object_oriented_a.pdf</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr">
@@ -5353,6 +5824,11 @@
       <c r="K93" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5870,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0071_modelling_and_analysis_of_distributed_software_using.pdf</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -5405,6 +5881,11 @@
       <c r="K94" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5449,9 +5930,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M95" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5974,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0054_decomposed_replay_using_hiding_and_reduction.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0054_decomposed_replay_using_hiding_and_reduction.pdf</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -5499,6 +5985,11 @@
       <c r="K96" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5540,7 +6031,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0101_effects_of_architecture_and_technical_development_pr.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0101_effects_of_architecture_and_technical_development_pr.pdf</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -5551,6 +6042,11 @@
       <c r="K97" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5592,7 +6088,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0093_calculating_the_usage_probabilities_of_statistical_u.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0093_calculating_the_usage_probabilities_of_statistical_u.pdf</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -5603,6 +6099,11 @@
       <c r="K98" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5657,9 +6158,14 @@
           <t>article</t>
         </is>
       </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M99" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -5699,9 +6205,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M100" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -5743,7 +6254,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0092_warnings_violation_symptoms_indicating_architecture.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0092_warnings_violation_symptoms_indicating_architecture.pdf</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -5754,6 +6265,11 @@
       <c r="K101" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5793,6 +6309,16 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="64" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
@@ -5830,9 +6356,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M103" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -5882,9 +6413,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M104" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -5926,7 +6462,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0058_reliability_of_task_execution_during_safe_software_p.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0058_reliability_of_task_execution_during_safe_software_p.pdf</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -5937,6 +6473,11 @@
       <c r="K105" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -5973,7 +6514,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0155_kanban_and_process_mining_in_the_task_management.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0155_kanban_and_process_mining_in_the_task_management.pdf</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -5984,6 +6525,11 @@
       <c r="K106" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6571,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0016_understanding_knowlegde_intensive_processes_from_tra.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0016_understanding_knowlegde_intensive_processes_from_tra.pdf</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -6036,6 +6582,11 @@
       <c r="K107" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6623,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0094_software_engineering_data_analysis_techniques.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0094_software_engineering_data_analysis_techniques.pdf</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -6083,6 +6634,11 @@
       <c r="K108" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6127,6 +6683,16 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="110" hidden="1" ht="320" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
@@ -6166,7 +6732,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0061_modeling_extraneous_activity_delays_in_business_proc.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0061_modeling_extraneous_activity_delays_in_business_proc.pdf</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -6177,6 +6743,11 @@
       <c r="K110" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -6231,6 +6802,16 @@
           <t>article</t>
         </is>
       </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="320" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
@@ -6273,9 +6854,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -6330,6 +6916,16 @@
           <t>article</t>
         </is>
       </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="114" hidden="1" ht="240" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
@@ -6369,7 +6965,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0017_reconstructing_meaningful_workflow_from_transaction.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0017_reconstructing_meaningful_workflow_from_transaction.pdf</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -6380,6 +6976,11 @@
       <c r="K114" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -6421,7 +7022,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0015_automated_generation_of_test_cases_using_a_performab.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0015_automated_generation_of_test_cases_using_a_performab.pdf</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -6432,6 +7033,11 @@
       <c r="K115" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6468,7 +7074,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0055_markovian_reliability_analysis_for_software_using_er.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0055_markovian_reliability_analysis_for_software_using_er.pdf</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -6479,6 +7085,11 @@
       <c r="K116" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
       <c r="M116" s="2" t="inlineStr">
@@ -6528,9 +7139,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M117" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -6567,7 +7183,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0073_software_performance_analysis_using_a_language_measu.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0073_software_performance_analysis_using_a_language_measu.pdf</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -6578,6 +7194,11 @@
       <c r="K118" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6632,9 +7253,14 @@
           <t>article</t>
         </is>
       </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M119" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -6676,7 +7302,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0121_quantitative_analysis_of_services.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0121_quantitative_analysis_of_services.pdf</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -6687,6 +7313,11 @@
       <c r="K120" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6723,7 +7354,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0112_an_extended_compdepend_algorithm_to_discovery_duplic.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0112_an_extended_compdepend_algorithm_to_discovery_duplic.pdf</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -6734,6 +7365,11 @@
       <c r="K121" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6775,7 +7411,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0106_simplifying_software_metric_models_via_hierarchical.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0106_simplifying_software_metric_models_via_hierarchical.pdf</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -6786,6 +7422,11 @@
       <c r="K122" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -6827,7 +7468,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0082_event_logs_for_the_analysis_of_software_failures_a_r.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0082_event_logs_for_the_analysis_of_software_failures_a_r.pdf</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr">
@@ -6838,6 +7479,11 @@
       <c r="K123" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6879,7 +7525,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0056_a_business_process_simulation_method_supporting_reso.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0056_a_business_process_simulation_method_supporting_reso.pdf</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -6890,6 +7536,11 @@
       <c r="K124" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6931,7 +7582,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0013_an_empirical_analysis_of_build_failures_in_the_conti.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0013_an_empirical_analysis_of_build_failures_in_the_conti.pdf</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -6942,6 +7593,11 @@
       <c r="K125" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -6983,7 +7639,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0170_monte_carlo_simulation_based_estimations_case_from_a.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0170_monte_carlo_simulation_based_estimations_case_from_a.pdf</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -6994,6 +7650,11 @@
       <c r="K126" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7030,7 +7691,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0171_the_economic_impact_of_software_process_variations.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0171_the_economic_impact_of_software_process_variations.pdf</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -7041,6 +7702,11 @@
       <c r="K127" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7077,7 +7743,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0150_nirikshan_process_mining_software_repositories_to_id.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0150_nirikshan_process_mining_software_repositories_to_id.pdf</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -7088,6 +7754,11 @@
       <c r="K128" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7124,7 +7795,7 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0167_monitoring_the_software_development_process_with_p.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0167_monitoring_the_software_development_process_with_p.pdf</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr">
@@ -7135,6 +7806,11 @@
       <c r="K129" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -7189,9 +7865,14 @@
           <t>article</t>
         </is>
       </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M130" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -7238,7 +7919,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0122_a_markov_error_propagation_model_for_component_based.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0122_a_markov_error_propagation_model_for_component_based.pdf</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -7249,6 +7930,11 @@
       <c r="K131" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7285,7 +7971,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0165_linking_software_process_modeling_with_markov_decisi.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0165_linking_software_process_modeling_with_markov_decisi.pdf</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -7296,6 +7982,11 @@
       <c r="K132" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7327,7 +8018,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0143_application_of_process_mining_in_project_management.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0143_application_of_process_mining_in_project_management.pdf</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr">
@@ -7338,6 +8029,11 @@
       <c r="K133" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7379,7 +8075,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0149_automatic_real_time_mining_software_process_activi.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0149_automatic_real_time_mining_software_process_activi.pdf</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -7390,6 +8086,11 @@
       <c r="K134" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7421,7 +8122,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0084_cross_company_collaboration_analyzed_through_process.pdf</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr">
@@ -7432,6 +8133,11 @@
       <c r="K135" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7468,7 +8174,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0077_the_use_of_knapsack_0_1_in_prioritizing_software_r.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0077_the_use_of_knapsack_0_1_in_prioritizing_software_r.pdf</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -7479,6 +8185,11 @@
       <c r="K136" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -7515,7 +8226,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0160_assessing_agile_software_development_processes_wit.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0160_assessing_agile_software_development_processes_wit.pdf</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -7526,6 +8237,11 @@
       <c r="K137" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7567,7 +8283,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0011_stochastic_aware_precision_and_recall_measures_for_c.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0011_stochastic_aware_precision_and_recall_measures_for_c.pdf</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -7578,6 +8294,11 @@
       <c r="K138" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7617,9 +8338,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M139" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -7656,7 +8382,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0098_a_hybrid_approach_to_process_mining_finding_immediat.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0098_a_hybrid_approach_to_process_mining_finding_immediat.pdf</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -7667,6 +8393,11 @@
       <c r="K140" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7713,7 +8444,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0166_applying_process_mining_the_reality_of_a_software_.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0166_applying_process_mining_the_reality_of_a_software_.pdf</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -7724,6 +8455,11 @@
       <c r="K141" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7765,7 +8501,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0039_a_vector_markov_model_for_structural_coverage_growth.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0039_a_vector_markov_model_for_structural_coverage_growth.pdf</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -7776,6 +8512,11 @@
       <c r="K142" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7815,9 +8556,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M143" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -7867,9 +8613,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M144" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -7916,7 +8667,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0139_discovery_and_simulation_of_data_aware_business_pr.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0139_discovery_and_simulation_of_data_aware_business_pr.pdf</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -7927,6 +8678,11 @@
       <c r="K145" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -7966,9 +8722,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M146" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -7998,9 +8759,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M147" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -8037,7 +8803,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0152_a_data_centric_approach_to_evaluate_requirements_e.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0152_a_data_centric_approach_to_evaluate_requirements_e.pdf</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -8048,6 +8814,11 @@
       <c r="K148" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8084,7 +8855,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0070_towards_goal_oriented_conformance_checking.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0070_towards_goal_oriented_conformance_checking.pdf</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
@@ -8095,6 +8866,11 @@
       <c r="K149" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8139,9 +8915,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M150" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8964,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0151_a_csp_theoretic_framework_of_checking_conformance_of.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0151_a_csp_theoretic_framework_of_checking_conformance_of.pdf</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -8194,6 +8975,11 @@
       <c r="K151" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -8235,7 +9021,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0105_an_approach_for_face_validity_assessment_of_agent_.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0105_an_approach_for_face_validity_assessment_of_agent_.pdf</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -8246,6 +9032,11 @@
       <c r="K152" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8295,9 +9086,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M153" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -8334,7 +9130,7 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0081_interactive_creation_visualization_and_exploration.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0081_interactive_creation_visualization_and_exploration.pdf</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr">
@@ -8345,6 +9141,11 @@
       <c r="K154" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -8386,7 +9187,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0146_a_method_for_stochastic_modeling_the_software_develo.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0146_a_method_for_stochastic_modeling_the_software_develo.pdf</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -8397,6 +9198,11 @@
       <c r="K155" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -8433,7 +9239,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0000_colored_petri_nets_simulation_on_the_cloud_with_pyth.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0000_colored_petri_nets_simulation_on_the_cloud_with_pyth.pdf</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -8444,6 +9250,11 @@
       <c r="K156" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8480,7 +9291,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0163_monitoring_a_ci_cd_workflow_using_process_mining.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0163_monitoring_a_ci_cd_workflow_using_process_mining.pdf</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">
@@ -8491,6 +9302,11 @@
       <c r="K157" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8532,7 +9348,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0050_architecture_of_process_mining_based_business_proces.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0050_architecture_of_process_mining_based_business_proces.pdf</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -8543,6 +9359,11 @@
       <c r="K158" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8589,7 +9410,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0021_discovering_simulation_models.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0021_discovering_simulation_models.pdf</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -8600,6 +9421,11 @@
       <c r="K159" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8641,7 +9467,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0168_process_mining_framework_for_software_processes.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0168_process_mining_framework_for_software_processes.pdf</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -8652,6 +9478,11 @@
       <c r="K160" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8688,7 +9519,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0173_predicting_issue_handling_process_using_case_attri.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0173_predicting_issue_handling_process_using_case_attri.pdf</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -8699,6 +9530,11 @@
       <c r="K161" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8745,7 +9581,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0046_remaining_activity_sequence_prediction_for_ongoing.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0046_remaining_activity_sequence_prediction_for_ongoing.pdf</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -8756,6 +9592,11 @@
       <c r="K162" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8810,9 +9651,14 @@
           <t>review</t>
         </is>
       </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M163" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -8852,9 +9698,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M164" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -8891,7 +9742,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0157_detecting_bottleneck_and_fraud_in_agile_developmen.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0157_detecting_bottleneck_and_fraud_in_agile_developmen.pdf</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -8902,6 +9753,11 @@
       <c r="K165" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8943,7 +9799,7 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0028_generating_transition_probabilities_for_automatic_mo.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0028_generating_transition_probabilities_for_automatic_mo.pdf</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -8954,6 +9810,11 @@
       <c r="K166" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -8998,9 +9859,14 @@
           <t>conference paper</t>
         </is>
       </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
       <c r="M167" s="2" t="inlineStr">
         <is>
-          <t>no access file</t>
+          <t>PDF não acessível</t>
         </is>
       </c>
     </row>
@@ -9037,7 +9903,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0118_stochastic_actor_oriented_modeling_for_studying_homo.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0118_stochastic_actor_oriented_modeling_for_studying_homo.pdf</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -9048,6 +9914,11 @@
       <c r="K168" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9950,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0104_simod_a_tool_for_automated_discovery_of_business_pro.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0104_simod_a_tool_for_automated_discovery_of_business_pro.pdf</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -9090,6 +9961,11 @@
       <c r="K169" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -9131,7 +10007,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0137_the_review_linkage_graph_for_code_review_analytics_a.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0137_the_review_linkage_graph_for_code_review_analytics_a.pdf</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr">
@@ -9142,6 +10018,11 @@
       <c r="K170" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -9188,7 +10069,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0044_software_reliability_modelling_and_prediction_with_h.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0044_software_reliability_modelling_and_prediction_with_h.pdf</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr">
@@ -9199,6 +10080,11 @@
       <c r="K171" s="2" t="inlineStr">
         <is>
           <t>article</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -9253,6 +10139,16 @@
           <t>article</t>
         </is>
       </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>PDF não acessível</t>
+        </is>
+      </c>
     </row>
     <row r="173" hidden="1" ht="16" customHeight="1">
       <c r="A173" s="2" t="inlineStr">
@@ -9282,7 +10178,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0066_mining_reuse_processes.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0066_mining_reuse_processes.pdf</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -9293,6 +10189,11 @@
       <c r="K173" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -9329,7 +10230,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0062_intelligent_agile_method_framework.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0062_intelligent_agile_method_framework.pdf</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
@@ -9340,6 +10241,11 @@
       <c r="K174" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -9381,7 +10287,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0023_optimal_test_profile_in_the_context_of_software_cybe.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0023_optimal_test_profile_in_the_context_of_software_cybe.pdf</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr">
@@ -9392,6 +10298,11 @@
       <c r="K175" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -9423,7 +10334,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0041_static_and_dynamic_architecture_conformance_checking.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0041_static_and_dynamic_architecture_conformance_checking.pdf</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr">
@@ -9434,6 +10345,11 @@
       <c r="K176" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>include</t>
         </is>
       </c>
     </row>
@@ -9475,7 +10391,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0153_predicting_release_time_based_on_generalized_softwar.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/no-ok/ft_0153_predicting_release_time_based_on_generalized_softwar.pdf</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -9486,6 +10402,11 @@
       <c r="K177" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>exclude</t>
         </is>
       </c>
     </row>
@@ -9527,7 +10448,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>results/human_validation/ft_pdfs_local/ft_0009_automated_method_for_verification_of_stochastic_grap.pdf</t>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0009_automated_method_for_verification_of_stochastic_grap.pdf</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr">
@@ -9538,6 +10459,126 @@
       <c r="K178" s="2" t="inlineStr">
         <is>
           <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>ft_0177</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Generating Hidden Markov Models from Process Models Through Nonnegative Tensor Factorization</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Skau E., Hollis A., Eidenbenz S., Rasmussen K., Alexandrov B.</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Monitoring of industrial processes is a critical capability in industry and in government to ensure reliability of production cycles, quick emergency response, and national security. We introduce a novel mathematically sound method that integrates theoretical process models with interrelated minimal Hidden Markov Models (HMM), built via nonnegative tensor factorization. Our method consolidates: (a) theoretical process models, (b) HMMs, (c) coupled nonnegative matrix-tensor factorizations, and (d) custom model selection. We apply it on simple synthetic and real-world process models.</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>10.1145/3664813</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3664813</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0177_generating_hidden_markov_models_from_process_models.pdf</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>ACM Transactions on Modeling and Computer Simulation (TOMACS), Vol 34, No 4, Article 21</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>article</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Adicionado via snowballing em 2026-08-13; nao estava no corpus Scopus original.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>ft_0178</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Discovery of Functional Architectures From Event Logs</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>van der Werf J.M.E.M., Kaats E.</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>The functional architecture focuses on decomposing functionality into modules that offer certain features, which require interactions to complete their functionality. This paper investigates the use of process discovery techniques to discover from scenarios the internal behavior of individual components. Based on event logs, this paper presents an approach (1) to derive the information flows between features, (2) identify the internal behavior of features, and (3) to discover the order between features within a module. The approach results in a sound workflow model for each module, illustrated using a running example of a payment system.</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>http://ceur-ws.org/Vol-1372/</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>results/human_validation/ft_pdfs_local/ok/ft_0178_discovery_of_functional_architectures_from_event_log.pdf</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>CEUR Workshop Proceedings Vol. 1372 - Proceedings of the International Workshop on Petri Nets and Software Engineering (PNSE'15)</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>conference paper</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Capitulo extraido do volume completo de anais (paginas 227-244 do PDF original, mantido como REFERENCE_pnse15_full_proceedings_vol1372.pdf na mesma pasta). Adicionado via snowballing em 2026-08-13.</t>
         </is>
       </c>
     </row>

</xml_diff>